<commit_message>
chore: sync .claude/skills install copies, add fresh-eyes-auditor skill
- Run scripts/check_skill_sync.py --apply to propagate all_skills/ canonical updates
  (rd/ paths, evaluation_plan.md rename, Rule 10 reports/ conventions) into .claude/skills/
- Install .claude/skills/ copies for previously canonical-only skills
  (context-engineering, dashboard-designer, defense-*, exp-runner, theory-decomposer,
  travel-planner-html, defense-proposal-assembler)
- Remove duplicate reference/examples files under .claude/skills/uf-chain-validator
  and .claude/skills/uf-if-debug-mapper to match canonical
- Add fresh-eyes-auditor skill (spawns context-free agent to audit ambiguity/forced-logic/
  errors/hallucination, triages findings by citation check; advisory, non-blocking)
- Update README.md and Skill_Combination_Usage_Guide.md to reference fresh-eyes-auditor
- Update uf-if-debug-mapper output path: debug_map.md -> docs/uf_if_debug_map.md

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/0.FilesUpdate.xlsx
+++ b/0.FilesUpdate.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -773,6 +773,23 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-07-21 11:40</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>all_skills/core-engineering_pipeline_skills/fresh-eyes-auditor/ (신규 3파일)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>무맥락 에이전트 4축 감사 스킬 (스폰 템플릿·트리아지·자문 리포트) + README/가이드 등재 + save_skill 계정 설치</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>